<commit_message>
update data file map
</commit_message>
<xml_diff>
--- a/DATA_FILE_MAP.xlsx
+++ b/DATA_FILE_MAP.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,7 +454,6 @@
           <t>life_sciences_main</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -472,7 +476,6 @@
           <t>look_west_media</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -495,7 +498,6 @@
           <t>look_west_funding</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>TRUE</t>

</xml_diff>

<commit_message>
Add policy table and pagination enhancements to Look West dashboard
</commit_message>
<xml_diff>
--- a/DATA_FILE_MAP.xlsx
+++ b/DATA_FILE_MAP.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,30 @@
           <t>Enter local synced SharePoint path</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>look_west_policy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Look West policy/regulations workbook</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Enter local file path</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
major projects + restructuring data folder
</commit_message>
<xml_diff>
--- a/DATA_FILE_MAP.xlsx
+++ b/DATA_FILE_MAP.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="FILE_MAP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILE_MAP" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,6 +454,11 @@
           <t>life_sciences_main</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dashboards/sectors/life_sciences/data/Life_Sciences_light.xlsx</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -520,7 +525,6 @@
           <t>look_west_policy</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -536,7 +540,6 @@
           <t>Enter local file path</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>